<commit_message>
Add R8 collection calendar and update property workbook
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換_列移動_20260513_計量リンク.xlsx
+++ b/2026年度物件表_KMN置換_列移動_20260513_計量リンク.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annsyuu/Desktop/CLAUDECODE計量物件表 （260404）/計量物件表の作成作業（Soft_Keiryou）/Keiryou_Editor/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annsyuu/Desktop/uenoseisou2.3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{AF69A894-7201-BF43-8995-1C83BFACAE25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{58A4D418-308F-A746-A62B-854CEF5AC799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="1280" windowWidth="28640" windowHeight="18020" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4540" yWindow="1280" windowWidth="28200" windowHeight="18020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026年度担当者物件表  20260127" sheetId="1" r:id="rId1"/>
@@ -4215,17 +4215,6 @@
     <xf numFmtId="0" fontId="37" fillId="17" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4242,6 +4231,17 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="スタイル 1" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -23527,91 +23527,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="263" t="s">
+      <c r="A1" s="258" t="s">
         <v>765</v>
       </c>
-      <c r="B1" s="264" t="s">
+      <c r="B1" s="259" t="s">
         <v>766</v>
       </c>
-      <c r="C1" s="265" t="s">
+      <c r="C1" s="260" t="s">
         <v>767</v>
       </c>
-      <c r="D1" s="265" t="s">
+      <c r="D1" s="260" t="s">
         <v>767</v>
       </c>
-      <c r="E1" s="265" t="s">
+      <c r="E1" s="260" t="s">
         <v>767</v>
       </c>
-      <c r="F1" s="265" t="s">
+      <c r="F1" s="260" t="s">
         <v>767</v>
       </c>
-      <c r="G1" s="265" t="s">
+      <c r="G1" s="260" t="s">
         <v>767</v>
       </c>
-      <c r="H1" s="265"/>
-      <c r="I1" s="265" t="s">
+      <c r="H1" s="260"/>
+      <c r="I1" s="260" t="s">
         <v>765</v>
       </c>
-      <c r="J1" s="265" t="s">
+      <c r="J1" s="260" t="s">
         <v>766</v>
       </c>
-      <c r="K1" s="265" t="s">
+      <c r="K1" s="260" t="s">
         <v>767</v>
       </c>
-      <c r="L1" s="265" t="s">
+      <c r="L1" s="260" t="s">
         <v>767</v>
       </c>
-      <c r="M1" s="265" t="s">
+      <c r="M1" s="260" t="s">
         <v>767</v>
       </c>
-      <c r="N1" s="265" t="s">
+      <c r="N1" s="260" t="s">
         <v>767</v>
       </c>
-      <c r="O1" s="265" t="s">
+      <c r="O1" s="260" t="s">
         <v>767</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="19.25" customHeight="1">
-      <c r="A2" s="260" t="s">
+      <c r="A2" s="255" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="261" t="s">
+      <c r="B2" s="256" t="s">
         <v>597</v>
       </c>
-      <c r="C2" s="261">
-        <v>1</v>
-      </c>
-      <c r="D2" s="261">
-        <v>2</v>
-      </c>
-      <c r="E2" s="261">
-        <v>3</v>
-      </c>
-      <c r="F2" s="261">
+      <c r="C2" s="256">
+        <v>1</v>
+      </c>
+      <c r="D2" s="256">
+        <v>2</v>
+      </c>
+      <c r="E2" s="256">
+        <v>3</v>
+      </c>
+      <c r="F2" s="256">
         <v>4</v>
       </c>
-      <c r="G2" s="262">
+      <c r="G2" s="257">
         <v>5</v>
       </c>
-      <c r="I2" s="260" t="s">
+      <c r="I2" s="255" t="s">
         <v>598</v>
       </c>
-      <c r="J2" s="261" t="s">
+      <c r="J2" s="256" t="s">
         <v>268</v>
       </c>
-      <c r="K2" s="261">
-        <v>1</v>
-      </c>
-      <c r="L2" s="261">
-        <v>2</v>
-      </c>
-      <c r="M2" s="261">
-        <v>3</v>
-      </c>
-      <c r="N2" s="261">
+      <c r="K2" s="256">
+        <v>1</v>
+      </c>
+      <c r="L2" s="256">
+        <v>2</v>
+      </c>
+      <c r="M2" s="256">
+        <v>3</v>
+      </c>
+      <c r="N2" s="256">
         <v>4</v>
       </c>
-      <c r="O2" s="262">
+      <c r="O2" s="257">
         <v>5</v>
       </c>
     </row>
@@ -36169,12 +36169,12 @@
       <c r="D22" s="245" t="s">
         <v>6</v>
       </c>
-      <c r="F22" s="255" t="s">
+      <c r="F22" s="261" t="s">
         <v>716</v>
       </c>
-      <c r="G22" s="256"/>
-      <c r="H22" s="256"/>
-      <c r="I22" s="257"/>
+      <c r="G22" s="262"/>
+      <c r="H22" s="262"/>
+      <c r="I22" s="263"/>
     </row>
     <row r="23" spans="1:10" ht="26.5" customHeight="1">
       <c r="A23" s="104">
@@ -37120,13 +37120,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="166" customFormat="1" ht="65" customHeight="1">
-      <c r="A1" s="258" t="s">
+      <c r="A1" s="264" t="s">
         <v>748</v>
       </c>
-      <c r="B1" s="259"/>
-      <c r="C1" s="259"/>
-      <c r="D1" s="259"/>
-      <c r="E1" s="259"/>
+      <c r="B1" s="265"/>
+      <c r="C1" s="265"/>
+      <c r="D1" s="265"/>
+      <c r="E1" s="265"/>
     </row>
     <row r="2" spans="1:5" s="166" customFormat="1" ht="36.5" customHeight="1">
       <c r="A2" s="188"/>

</xml_diff>